<commit_message>
record three reported full-text updates
</commit_message>
<xml_diff>
--- a/系统评价_最终英文投稿交付版/189条全文批量获取清单.xlsx
+++ b/系统评价_最终英文投稿交付版/189条全文批量获取清单.xlsx
@@ -1780,17 +1780,17 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>网络访问失败</t>
+          <t>已获取（用户报告；本工作区未核验PDF）</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>NO_METADATA_MATCH</t>
+          <t>Record_ID由用户提供；全文文件身份待核验</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>OpenAlex: OpenAlex disabled after a prior 403/proxy/network failure | Europe PMC: Europe PMC disabled after a prior 403/proxy/network failure</t>
+          <t>用户在对话提供的全文进度表；未提供PDF文件或来源链接</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
@@ -1800,14 +1800,26 @@
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27 11:54 UTC</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="V12" s="2" t="n"/>
       <c r="W12" s="2" t="n"/>
-      <c r="X12" s="2" t="n"/>
-      <c r="Y12" s="2" t="n"/>
-      <c r="Z12" s="2" t="n"/>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>PENDING：用户未提供</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>PENDING：当前工作区未见对应PDF</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>NOT_VERIFIED_LOCALLY</t>
+        </is>
+      </c>
       <c r="AA12" s="2" t="n"/>
     </row>
     <row r="13">
@@ -10335,17 +10347,17 @@
       </c>
       <c r="Q91" s="2" t="inlineStr">
         <is>
-          <t>网络访问失败</t>
+          <t>已获取（用户报告；本工作区未核验PDF）</t>
         </is>
       </c>
       <c r="R91" s="2" t="inlineStr">
         <is>
-          <t>NO_METADATA_MATCH</t>
+          <t>Record_ID由用户提供；全文文件身份待核验</t>
         </is>
       </c>
       <c r="S91" s="2" t="inlineStr">
         <is>
-          <t>OpenAlex: OpenAlex disabled after a prior 403/proxy/network failure | Europe PMC: Europe PMC disabled after a prior 403/proxy/network failure</t>
+          <t>用户在对话提供的全文进度表；未提供PDF文件或来源链接</t>
         </is>
       </c>
       <c r="T91" s="2" t="inlineStr">
@@ -10355,14 +10367,26 @@
       </c>
       <c r="U91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27 11:54 UTC</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="V91" s="2" t="n"/>
       <c r="W91" s="2" t="n"/>
-      <c r="X91" s="2" t="n"/>
-      <c r="Y91" s="2" t="n"/>
-      <c r="Z91" s="2" t="n"/>
+      <c r="X91" s="2" t="inlineStr">
+        <is>
+          <t>PENDING：用户未提供</t>
+        </is>
+      </c>
+      <c r="Y91" s="2" t="inlineStr">
+        <is>
+          <t>PENDING：当前工作区未见对应PDF</t>
+        </is>
+      </c>
+      <c r="Z91" s="2" t="inlineStr">
+        <is>
+          <t>NOT_VERIFIED_LOCALLY</t>
+        </is>
+      </c>
       <c r="AA91" s="2" t="n"/>
     </row>
     <row r="92">
@@ -20546,17 +20570,17 @@
       </c>
       <c r="Q186" s="2" t="inlineStr">
         <is>
-          <t>网络访问失败</t>
+          <t>已获取（用户报告；本工作区未核验PDF）</t>
         </is>
       </c>
       <c r="R186" s="2" t="inlineStr">
         <is>
-          <t>NO_METADATA_MATCH</t>
+          <t>Record_ID由用户提供；全文文件身份待核验</t>
         </is>
       </c>
       <c r="S186" s="2" t="inlineStr">
         <is>
-          <t>OpenAlex: OpenAlex disabled after a prior 403/proxy/network failure | Europe PMC: Europe PMC disabled after a prior 403/proxy/network failure</t>
+          <t>用户在对话提供的全文进度表；未提供PDF文件或来源链接</t>
         </is>
       </c>
       <c r="T186" s="2" t="inlineStr">
@@ -20566,14 +20590,26 @@
       </c>
       <c r="U186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27 11:55 UTC</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="V186" s="2" t="n"/>
       <c r="W186" s="2" t="n"/>
-      <c r="X186" s="2" t="n"/>
-      <c r="Y186" s="2" t="n"/>
-      <c r="Z186" s="2" t="n"/>
+      <c r="X186" s="2" t="inlineStr">
+        <is>
+          <t>PENDING：用户未提供</t>
+        </is>
+      </c>
+      <c r="Y186" s="2" t="inlineStr">
+        <is>
+          <t>PENDING：当前工作区未见对应PDF</t>
+        </is>
+      </c>
+      <c r="Z186" s="2" t="inlineStr">
+        <is>
+          <t>NOT_VERIFIED_LOCALLY</t>
+        </is>
+      </c>
       <c r="AA186" s="2" t="n"/>
     </row>
     <row r="187">

</xml_diff>